<commit_message>
Redesign RQ5 v1 blind packets for construct-valid necessity judgments.
Replace generic pytest briefs and substring [[REF]] corruption with snapshot-derived tasks, minimal repo context, semantic path redaction, translation, and fail-closed exclusions.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/rq5_lb_blind_annotation/human_annotation_kit/ANNOTATION_FORM.xlsx
+++ b/exports/rq5_lb_blind_annotation/human_annotation_kit/ANNOTATION_FORM.xlsx
@@ -270,7 +270,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4b9a3c6654895937</t>
+          <t>5cdb19823812fea3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -302,7 +302,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5cdb19823812fea3</t>
+          <t>67c2974c57527180</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -334,7 +334,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>67c2974c57527180</t>
+          <t>8222c534ec20c9c2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -366,7 +366,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>80994240f7b369b7</t>
+          <t>85571219ad372807</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -398,7 +398,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8222c534ec20c9c2</t>
+          <t>8819745939ade378</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -430,7 +430,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>85571219ad372807</t>
+          <t>8a7005d04252096c</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -462,7 +462,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8819745939ade378</t>
+          <t>8bec66320d554a6d</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8a7005d04252096c</t>
+          <t>91a44ede937683ce</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -526,7 +526,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8bec66320d554a6d</t>
+          <t>91ecefdc5a31edaf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -558,7 +558,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>91a44ede937683ce</t>
+          <t>a38973860e5d4712</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -590,7 +590,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>91ecefdc5a31edaf</t>
+          <t>ac63aa4470fd018b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>930e6bd912075b0c</t>
+          <t>b6f1d2c6e3328de2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -654,7 +654,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>a38973860e5d4712</t>
+          <t>b8695a2837b8211e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -686,7 +686,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ac63aa4470fd018b</t>
+          <t>be858faa4705fb53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -718,7 +718,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>b6f1d2c6e3328de2</t>
+          <t>c7ee59d30924c48f</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -750,7 +750,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>b8695a2837b8211e</t>
+          <t>d6f94af612431129</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>be858faa4705fb53</t>
+          <t>e2642ac6cb4568a4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -806,230 +806,6 @@
         </is>
       </c>
       <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>c7ee59d30924c48f</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>cbea9e122bb3ae2f</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>d6f94af612431129</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>e2642ac6cb4568a4</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>edc493748044c205</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>fa72bc285f4b7183</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>faa505ff151a1867</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>